<commit_message>
Hapus kolom L/P dari template dan UI (tidak dibutuhkan checker)
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/template_data_mahasiswa.xlsx
+++ b/static/template_data_mahasiswa.xlsx
@@ -444,14 +444,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,11 +471,6 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>L/P</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
           <t>PERGURUAN TINGGI</t>
         </is>
       </c>
@@ -495,12 +489,7 @@
           <t>AHMAD SANDI</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>UNIVERSITAS TADULAKO</t>
         </is>
@@ -520,12 +509,7 @@
           <t>HABIBA</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>UNIVERSITAS HALU OLEO</t>
         </is>
@@ -537,8 +521,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr"/>
       <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -546,8 +529,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr"/>
       <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -555,8 +537,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr"/>
       <c r="C6" s="3" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>